<commit_message>
modelo de boca y estomago con ecuaciones
</commit_message>
<xml_diff>
--- a/Datos generales digestion.xlsx
+++ b/Datos generales digestion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\heber\Desktop\proyecto 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B54C31A1-4364-4C9D-ACE9-2664A997856D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C242D413-8602-4C0B-8A58-0EF28DD722FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{A64F9E11-6710-4C33-9930-3773814F4B53}"/>
   </bookViews>
@@ -207,7 +207,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -219,6 +219,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -847,7 +853,7 @@
         <v>37</v>
       </c>
       <c r="H8" s="3">
-        <v>25.42</v>
+        <v>26.42</v>
       </c>
       <c r="I8" s="3">
         <v>0.161</v>
@@ -876,7 +882,7 @@
         <v>37</v>
       </c>
       <c r="H9" s="3">
-        <v>25.67</v>
+        <v>26.67</v>
       </c>
       <c r="I9" s="3">
         <v>0.14099999999999999</v>
@@ -905,7 +911,7 @@
         <v>37</v>
       </c>
       <c r="H10" s="3">
-        <v>25.65</v>
+        <v>26.65</v>
       </c>
       <c r="I10" s="3">
         <v>0.121</v>
@@ -934,7 +940,7 @@
         <v>37</v>
       </c>
       <c r="H11" s="3">
-        <v>26.48</v>
+        <v>25.48</v>
       </c>
       <c r="I11" s="3">
         <v>0.27300000000000002</v>
@@ -963,7 +969,7 @@
         <v>37</v>
       </c>
       <c r="H12" s="3">
-        <v>26.18</v>
+        <v>25.18</v>
       </c>
       <c r="I12" s="3">
         <v>0.218</v>
@@ -992,7 +998,7 @@
         <v>37</v>
       </c>
       <c r="H13" s="3">
-        <v>26.22</v>
+        <v>25.22</v>
       </c>
       <c r="I13" s="3">
         <v>0.247</v>
@@ -1695,6 +1701,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
cineticas de  boca, estomago e intestino
</commit_message>
<xml_diff>
--- a/Datos generales digestion.xlsx
+++ b/Datos generales digestion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\heber\Desktop\proyecto 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C242D413-8602-4C0B-8A58-0EF28DD722FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DD1BAB0-50BD-46F3-B4BA-8A50FD5F6C71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{A64F9E11-6710-4C33-9930-3773814F4B53}"/>
   </bookViews>
@@ -1027,7 +1027,7 @@
         <v>37</v>
       </c>
       <c r="H14" s="3">
-        <v>28.85</v>
+        <v>25.85</v>
       </c>
       <c r="I14" s="3">
         <v>0.129</v>
@@ -1114,7 +1114,7 @@
         <v>37</v>
       </c>
       <c r="H17" s="3">
-        <v>28.85</v>
+        <v>25.85</v>
       </c>
       <c r="I17" s="3">
         <v>0.105</v>
@@ -1201,7 +1201,7 @@
         <v>37</v>
       </c>
       <c r="H20" s="3">
-        <v>38.630000000000003</v>
+        <v>25.63</v>
       </c>
       <c r="I20" s="3">
         <v>8.5999999999999993E-2</v>
@@ -1375,7 +1375,7 @@
         <v>37</v>
       </c>
       <c r="H26" s="3">
-        <v>39.67</v>
+        <v>26.67</v>
       </c>
       <c r="I26" s="3">
         <v>8.7999999999999995E-2</v>
@@ -1491,7 +1491,7 @@
         <v>37</v>
       </c>
       <c r="H30" s="3">
-        <v>43.8</v>
+        <v>26.8</v>
       </c>
       <c r="I30" s="3">
         <v>0.19600000000000001</v>
@@ -1549,7 +1549,7 @@
         <v>37</v>
       </c>
       <c r="H32" s="3">
-        <v>25.73</v>
+        <v>26.73</v>
       </c>
       <c r="I32" s="3">
         <v>0.16800000000000001</v>
@@ -1636,7 +1636,7 @@
         <v>37</v>
       </c>
       <c r="H35" s="3">
-        <v>39.19</v>
+        <v>26.19</v>
       </c>
       <c r="I35" s="3">
         <v>0.10299999999999999</v>

</xml_diff>